<commit_message>
Phase 4: token optimization v3-5, ROI prediction, Gemini fix
- Token opt v3 (#22): 중간 표 제거·헤더 단순화 (~1,350토큰 절감)
- Token opt v4 (#1/#3/#5): label-map/ai-score-compare/parse-requirement 압축 (~800토큰)
- Token opt v5 D/E/F (#25): txt+JSON 병행구성·비선택안 단축·roi_calc 사전계산 (~750~1,000토큰+13~20초)
- ROI 예측 기능 (#23): roi-estimation-guide.md 신규, weekly_hours 파싱, Excel ROI 6필드
- Gemini CLI fix (#24): python3→py 수정 (Windows MS Store 리다이렉트 대응)
- Excel 저장 경로 변경: xlsx → output/ 직접 저장 (output/Archive/ 제외)
</commit_message>
<xml_diff>
--- a/Word_Template/컨설팅결과_보고서_템플릿.xlsx
+++ b/Word_Template/컨설팅결과_보고서_템플릿.xlsx
@@ -117,7 +117,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -192,6 +192,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F3E5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000695C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0F2F1"/>
       </patternFill>
     </fill>
   </fills>
@@ -314,7 +324,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -362,6 +372,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -426,6 +442,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -802,7 +824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:F73"/>
+  <dimension ref="A2:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -820,19 +842,19 @@
           <t>MS 업무 자동화  컨설팅 결과 보고서</t>
         </is>
       </c>
-      <c r="B2" s="20" t="n"/>
-      <c r="C2" s="20" t="n"/>
-      <c r="D2" s="20" t="n"/>
-      <c r="E2" s="20" t="n"/>
-      <c r="F2" s="21" t="n"/>
+      <c r="B2" s="22" t="n"/>
+      <c r="C2" s="22" t="n"/>
+      <c r="D2" s="22" t="n"/>
+      <c r="E2" s="22" t="n"/>
+      <c r="F2" s="23" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="22" t="n"/>
-      <c r="B3" s="23" t="n"/>
-      <c r="C3" s="23" t="n"/>
-      <c r="D3" s="23" t="n"/>
-      <c r="E3" s="23" t="n"/>
-      <c r="F3" s="24" t="n"/>
+      <c r="A3" s="24" t="n"/>
+      <c r="B3" s="25" t="n"/>
+      <c r="C3" s="25" t="n"/>
+      <c r="D3" s="25" t="n"/>
+      <c r="E3" s="25" t="n"/>
+      <c r="F3" s="26" t="n"/>
     </row>
     <row r="4" ht="6" customHeight="1"/>
     <row r="5" ht="24" customHeight="1">
@@ -1028,10 +1050,10 @@
           <t>{{REQ_CONSTRAINTS}}</t>
         </is>
       </c>
-      <c r="C15" s="25" t="n"/>
-      <c r="D15" s="25" t="n"/>
-      <c r="E15" s="25" t="n"/>
-      <c r="F15" s="26" t="n"/>
+      <c r="C15" s="27" t="n"/>
+      <c r="D15" s="27" t="n"/>
+      <c r="E15" s="27" t="n"/>
+      <c r="F15" s="28" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
@@ -1058,10 +1080,10 @@
           <t>{{SOL_REC_NAME}}</t>
         </is>
       </c>
-      <c r="C19" s="25" t="n"/>
-      <c r="D19" s="25" t="n"/>
-      <c r="E19" s="25" t="n"/>
-      <c r="F19" s="26" t="n"/>
+      <c r="C19" s="27" t="n"/>
+      <c r="D19" s="27" t="n"/>
+      <c r="E19" s="27" t="n"/>
+      <c r="F19" s="28" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
@@ -1074,10 +1096,10 @@
           <t>{{SOL_REC_REASON}}</t>
         </is>
       </c>
-      <c r="C20" s="25" t="n"/>
-      <c r="D20" s="25" t="n"/>
-      <c r="E20" s="25" t="n"/>
-      <c r="F20" s="26" t="n"/>
+      <c r="C20" s="27" t="n"/>
+      <c r="D20" s="27" t="n"/>
+      <c r="E20" s="27" t="n"/>
+      <c r="F20" s="28" t="n"/>
     </row>
     <row r="21" ht="40" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
@@ -1090,10 +1112,10 @@
           <t>{{SOL_REC_FLOW}}</t>
         </is>
       </c>
-      <c r="C21" s="25" t="n"/>
-      <c r="D21" s="25" t="n"/>
-      <c r="E21" s="25" t="n"/>
-      <c r="F21" s="26" t="n"/>
+      <c r="C21" s="27" t="n"/>
+      <c r="D21" s="27" t="n"/>
+      <c r="E21" s="27" t="n"/>
+      <c r="F21" s="28" t="n"/>
     </row>
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
@@ -1106,10 +1128,10 @@
           <t>{{SOL_REC_PREREQ}}</t>
         </is>
       </c>
-      <c r="C22" s="25" t="n"/>
-      <c r="D22" s="25" t="n"/>
-      <c r="E22" s="25" t="n"/>
-      <c r="F22" s="26" t="n"/>
+      <c r="C22" s="27" t="n"/>
+      <c r="D22" s="27" t="n"/>
+      <c r="E22" s="27" t="n"/>
+      <c r="F22" s="28" t="n"/>
     </row>
     <row r="23" ht="40" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
@@ -1122,10 +1144,10 @@
           <t>{{SOL_REC_CAUTION}}</t>
         </is>
       </c>
-      <c r="C23" s="25" t="n"/>
-      <c r="D23" s="25" t="n"/>
-      <c r="E23" s="25" t="n"/>
-      <c r="F23" s="26" t="n"/>
+      <c r="C23" s="27" t="n"/>
+      <c r="D23" s="27" t="n"/>
+      <c r="E23" s="27" t="n"/>
+      <c r="F23" s="28" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
@@ -1145,10 +1167,10 @@
           <t>{{SOL_REV_NAME}}</t>
         </is>
       </c>
-      <c r="C26" s="25" t="n"/>
-      <c r="D26" s="25" t="n"/>
-      <c r="E26" s="25" t="n"/>
-      <c r="F26" s="26" t="n"/>
+      <c r="C26" s="27" t="n"/>
+      <c r="D26" s="27" t="n"/>
+      <c r="E26" s="27" t="n"/>
+      <c r="F26" s="28" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
@@ -1161,10 +1183,10 @@
           <t>{{SOL_REV_REASON}}</t>
         </is>
       </c>
-      <c r="C27" s="25" t="n"/>
-      <c r="D27" s="25" t="n"/>
-      <c r="E27" s="25" t="n"/>
-      <c r="F27" s="26" t="n"/>
+      <c r="C27" s="27" t="n"/>
+      <c r="D27" s="27" t="n"/>
+      <c r="E27" s="27" t="n"/>
+      <c r="F27" s="28" t="n"/>
     </row>
     <row r="28" ht="40" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
@@ -1177,10 +1199,10 @@
           <t>{{SOL_REV_FLOW}}</t>
         </is>
       </c>
-      <c r="C28" s="25" t="n"/>
-      <c r="D28" s="25" t="n"/>
-      <c r="E28" s="25" t="n"/>
-      <c r="F28" s="26" t="n"/>
+      <c r="C28" s="27" t="n"/>
+      <c r="D28" s="27" t="n"/>
+      <c r="E28" s="27" t="n"/>
+      <c r="F28" s="28" t="n"/>
     </row>
     <row r="29" ht="40" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
@@ -1193,10 +1215,10 @@
           <t>{{SOL_REV_PREREQ}}</t>
         </is>
       </c>
-      <c r="C29" s="25" t="n"/>
-      <c r="D29" s="25" t="n"/>
-      <c r="E29" s="25" t="n"/>
-      <c r="F29" s="26" t="n"/>
+      <c r="C29" s="27" t="n"/>
+      <c r="D29" s="27" t="n"/>
+      <c r="E29" s="27" t="n"/>
+      <c r="F29" s="28" t="n"/>
     </row>
     <row r="30" ht="40" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
@@ -1209,10 +1231,10 @@
           <t>{{SOL_REV_CAUTION}}</t>
         </is>
       </c>
-      <c r="C30" s="25" t="n"/>
-      <c r="D30" s="25" t="n"/>
-      <c r="E30" s="25" t="n"/>
-      <c r="F30" s="26" t="n"/>
+      <c r="C30" s="27" t="n"/>
+      <c r="D30" s="27" t="n"/>
+      <c r="E30" s="27" t="n"/>
+      <c r="F30" s="28" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
@@ -1232,10 +1254,10 @@
           <t>{{SOL_NOT_NAME}}</t>
         </is>
       </c>
-      <c r="C33" s="25" t="n"/>
-      <c r="D33" s="25" t="n"/>
-      <c r="E33" s="25" t="n"/>
-      <c r="F33" s="26" t="n"/>
+      <c r="C33" s="27" t="n"/>
+      <c r="D33" s="27" t="n"/>
+      <c r="E33" s="27" t="n"/>
+      <c r="F33" s="28" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
@@ -1248,10 +1270,10 @@
           <t>{{SOL_NOT_REASON}}</t>
         </is>
       </c>
-      <c r="C34" s="25" t="n"/>
-      <c r="D34" s="25" t="n"/>
-      <c r="E34" s="25" t="n"/>
-      <c r="F34" s="26" t="n"/>
+      <c r="C34" s="27" t="n"/>
+      <c r="D34" s="27" t="n"/>
+      <c r="E34" s="27" t="n"/>
+      <c r="F34" s="28" t="n"/>
     </row>
     <row r="36" ht="24" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
@@ -1278,10 +1300,10 @@
           <t>{{SOL_REC_NAME}}  |  ID: {{SOL_REC_ID}}</t>
         </is>
       </c>
-      <c r="C38" s="25" t="n"/>
-      <c r="D38" s="25" t="n"/>
-      <c r="E38" s="25" t="n"/>
-      <c r="F38" s="26" t="n"/>
+      <c r="C38" s="27" t="n"/>
+      <c r="D38" s="27" t="n"/>
+      <c r="E38" s="27" t="n"/>
+      <c r="F38" s="28" t="n"/>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
@@ -1294,10 +1316,10 @@
           <t>{{SOL_REC_TECH_REASON}}</t>
         </is>
       </c>
-      <c r="C39" s="25" t="n"/>
-      <c r="D39" s="25" t="n"/>
-      <c r="E39" s="25" t="n"/>
-      <c r="F39" s="26" t="n"/>
+      <c r="C39" s="27" t="n"/>
+      <c r="D39" s="27" t="n"/>
+      <c r="E39" s="27" t="n"/>
+      <c r="F39" s="28" t="n"/>
     </row>
     <row r="40" ht="50" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
@@ -1310,10 +1332,10 @@
           <t>{{SOL_REC_IMPL_OVERVIEW}}</t>
         </is>
       </c>
-      <c r="C40" s="25" t="n"/>
-      <c r="D40" s="25" t="n"/>
-      <c r="E40" s="25" t="n"/>
-      <c r="F40" s="26" t="n"/>
+      <c r="C40" s="27" t="n"/>
+      <c r="D40" s="27" t="n"/>
+      <c r="E40" s="27" t="n"/>
+      <c r="F40" s="28" t="n"/>
     </row>
     <row r="41" ht="50" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
@@ -1326,10 +1348,10 @@
           <t>{{SOL_REC_PREREQ_TECH}}</t>
         </is>
       </c>
-      <c r="C41" s="25" t="n"/>
-      <c r="D41" s="25" t="n"/>
-      <c r="E41" s="25" t="n"/>
-      <c r="F41" s="26" t="n"/>
+      <c r="C41" s="27" t="n"/>
+      <c r="D41" s="27" t="n"/>
+      <c r="E41" s="27" t="n"/>
+      <c r="F41" s="28" t="n"/>
     </row>
     <row r="42" ht="50" customHeight="1">
       <c r="A42" s="3" t="inlineStr">
@@ -1342,10 +1364,10 @@
           <t>{{SOL_REC_LIMITS}}</t>
         </is>
       </c>
-      <c r="C42" s="25" t="n"/>
-      <c r="D42" s="25" t="n"/>
-      <c r="E42" s="25" t="n"/>
-      <c r="F42" s="26" t="n"/>
+      <c r="C42" s="27" t="n"/>
+      <c r="D42" s="27" t="n"/>
+      <c r="E42" s="27" t="n"/>
+      <c r="F42" s="28" t="n"/>
     </row>
     <row r="43" ht="50" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
@@ -1358,10 +1380,10 @@
           <t>{{SOL_REC_CONSIDERATIONS}}</t>
         </is>
       </c>
-      <c r="C43" s="25" t="n"/>
-      <c r="D43" s="25" t="n"/>
-      <c r="E43" s="25" t="n"/>
-      <c r="F43" s="26" t="n"/>
+      <c r="C43" s="27" t="n"/>
+      <c r="D43" s="27" t="n"/>
+      <c r="E43" s="27" t="n"/>
+      <c r="F43" s="28" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="3" t="inlineStr">
@@ -1386,16 +1408,8 @@
           <t>영향도</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>발생 조건</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>대응 방안</t>
-        </is>
-      </c>
+      <c r="C45" s="5" t="inlineStr"/>
+      <c r="D45" s="5" t="inlineStr"/>
       <c r="E45" s="5" t="inlineStr"/>
       <c r="F45" s="5" t="inlineStr"/>
     </row>
@@ -1415,13 +1429,13 @@
           <t>{{RISK_SEC_CONDITION}}</t>
         </is>
       </c>
-      <c r="D46" s="26" t="n"/>
+      <c r="D46" s="28" t="n"/>
       <c r="E46" s="4" t="inlineStr">
         <is>
           <t>{{RISK_SEC_ACTION}}</t>
         </is>
       </c>
-      <c r="F46" s="26" t="n"/>
+      <c r="F46" s="28" t="n"/>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
@@ -1439,13 +1453,13 @@
           <t>{{RISK_LIC_CONDITION}}</t>
         </is>
       </c>
-      <c r="D47" s="26" t="n"/>
+      <c r="D47" s="28" t="n"/>
       <c r="E47" s="4" t="inlineStr">
         <is>
           <t>{{RISK_LIC_ACTION}}</t>
         </is>
       </c>
-      <c r="F47" s="26" t="n"/>
+      <c r="F47" s="28" t="n"/>
     </row>
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
@@ -1463,13 +1477,13 @@
           <t>{{RISK_OPS_CONDITION}}</t>
         </is>
       </c>
-      <c r="D48" s="26" t="n"/>
+      <c r="D48" s="28" t="n"/>
       <c r="E48" s="4" t="inlineStr">
         <is>
           <t>{{RISK_OPS_ACTION}}</t>
         </is>
       </c>
-      <c r="F48" s="26" t="n"/>
+      <c r="F48" s="28" t="n"/>
     </row>
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
@@ -1489,10 +1503,10 @@
           <t>{{SOL_REV_NAME}}  |  ID: {{SOL_REV_ID}}</t>
         </is>
       </c>
-      <c r="C51" s="25" t="n"/>
-      <c r="D51" s="25" t="n"/>
-      <c r="E51" s="25" t="n"/>
-      <c r="F51" s="26" t="n"/>
+      <c r="C51" s="27" t="n"/>
+      <c r="D51" s="27" t="n"/>
+      <c r="E51" s="27" t="n"/>
+      <c r="F51" s="28" t="n"/>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="3" t="inlineStr">
@@ -1505,10 +1519,10 @@
           <t>{{SOL_REV_TECH_REASON}}</t>
         </is>
       </c>
-      <c r="C52" s="25" t="n"/>
-      <c r="D52" s="25" t="n"/>
-      <c r="E52" s="25" t="n"/>
-      <c r="F52" s="26" t="n"/>
+      <c r="C52" s="27" t="n"/>
+      <c r="D52" s="27" t="n"/>
+      <c r="E52" s="27" t="n"/>
+      <c r="F52" s="28" t="n"/>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
@@ -1521,10 +1535,10 @@
           <t>{{SOL_REV_JUDGMENT}}</t>
         </is>
       </c>
-      <c r="C53" s="25" t="n"/>
-      <c r="D53" s="25" t="n"/>
-      <c r="E53" s="25" t="n"/>
-      <c r="F53" s="26" t="n"/>
+      <c r="C53" s="27" t="n"/>
+      <c r="D53" s="27" t="n"/>
+      <c r="E53" s="27" t="n"/>
+      <c r="F53" s="28" t="n"/>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="11" t="inlineStr">
@@ -1544,10 +1558,10 @@
           <t>{{SOL_NOT_NAME}}  |  ID: {{SOL_NOT_ID}}</t>
         </is>
       </c>
-      <c r="C56" s="25" t="n"/>
-      <c r="D56" s="25" t="n"/>
-      <c r="E56" s="25" t="n"/>
-      <c r="F56" s="26" t="n"/>
+      <c r="C56" s="27" t="n"/>
+      <c r="D56" s="27" t="n"/>
+      <c r="E56" s="27" t="n"/>
+      <c r="F56" s="28" t="n"/>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="3" t="inlineStr">
@@ -1560,10 +1574,10 @@
           <t>{{SOL_NOT_TECH_REASON}}</t>
         </is>
       </c>
-      <c r="C57" s="25" t="n"/>
-      <c r="D57" s="25" t="n"/>
-      <c r="E57" s="25" t="n"/>
-      <c r="F57" s="26" t="n"/>
+      <c r="C57" s="27" t="n"/>
+      <c r="D57" s="27" t="n"/>
+      <c r="E57" s="27" t="n"/>
+      <c r="F57" s="28" t="n"/>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
@@ -1576,10 +1590,10 @@
           <t>{{SOL_NOT_JUDGMENT}}</t>
         </is>
       </c>
-      <c r="C58" s="25" t="n"/>
-      <c r="D58" s="25" t="n"/>
-      <c r="E58" s="25" t="n"/>
-      <c r="F58" s="26" t="n"/>
+      <c r="C58" s="27" t="n"/>
+      <c r="D58" s="27" t="n"/>
+      <c r="E58" s="27" t="n"/>
+      <c r="F58" s="28" t="n"/>
     </row>
     <row r="60" ht="24" customHeight="1">
       <c r="A60" s="15" t="inlineStr">
@@ -1599,10 +1613,10 @@
           <t>{{AI_OVERVIEW}}</t>
         </is>
       </c>
-      <c r="C61" s="25" t="n"/>
-      <c r="D61" s="25" t="n"/>
-      <c r="E61" s="25" t="n"/>
-      <c r="F61" s="26" t="n"/>
+      <c r="C61" s="27" t="n"/>
+      <c r="D61" s="27" t="n"/>
+      <c r="E61" s="27" t="n"/>
+      <c r="F61" s="28" t="n"/>
     </row>
     <row r="62" ht="50" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
@@ -1615,10 +1629,10 @@
           <t>{{AI_FINDINGS}}</t>
         </is>
       </c>
-      <c r="C62" s="25" t="n"/>
-      <c r="D62" s="25" t="n"/>
-      <c r="E62" s="25" t="n"/>
-      <c r="F62" s="26" t="n"/>
+      <c r="C62" s="27" t="n"/>
+      <c r="D62" s="27" t="n"/>
+      <c r="E62" s="27" t="n"/>
+      <c r="F62" s="28" t="n"/>
     </row>
     <row r="63" ht="50" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
@@ -1631,10 +1645,10 @@
           <t>{{AI_RECOMMENDATIONS}}</t>
         </is>
       </c>
-      <c r="C63" s="25" t="n"/>
-      <c r="D63" s="25" t="n"/>
-      <c r="E63" s="25" t="n"/>
-      <c r="F63" s="26" t="n"/>
+      <c r="C63" s="27" t="n"/>
+      <c r="D63" s="27" t="n"/>
+      <c r="E63" s="27" t="n"/>
+      <c r="F63" s="28" t="n"/>
     </row>
     <row r="64" ht="50" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
@@ -1647,191 +1661,299 @@
           <t>{{AI_EXTRA_RISK_OPP}}</t>
         </is>
       </c>
-      <c r="C64" s="25" t="n"/>
-      <c r="D64" s="25" t="n"/>
-      <c r="E64" s="25" t="n"/>
-      <c r="F64" s="26" t="n"/>
+      <c r="C64" s="27" t="n"/>
+      <c r="D64" s="27" t="n"/>
+      <c r="E64" s="27" t="n"/>
+      <c r="F64" s="28" t="n"/>
     </row>
     <row r="66" ht="24" customHeight="1">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5.  ROI 예측</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>현재 작업 시간</t>
+        </is>
+      </c>
+      <c r="B67" s="18" t="inlineStr">
+        <is>
+          <t>{{ROI_CURRENT_TIME}}</t>
+        </is>
+      </c>
+      <c r="C67" s="27" t="n"/>
+      <c r="D67" s="27" t="n"/>
+      <c r="E67" s="27" t="n"/>
+      <c r="F67" s="28" t="n"/>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>개선 후 예상 시간</t>
+        </is>
+      </c>
+      <c r="B68" s="18" t="inlineStr">
+        <is>
+          <t>{{ROI_IMPROVED_TIME}}</t>
+        </is>
+      </c>
+      <c r="C68" s="27" t="n"/>
+      <c r="D68" s="27" t="n"/>
+      <c r="E68" s="27" t="n"/>
+      <c r="F68" s="28" t="n"/>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>절감 효과</t>
+        </is>
+      </c>
+      <c r="B69" s="18" t="inlineStr">
+        <is>
+          <t>{{ROI_SAVE_PERIOD}}</t>
+        </is>
+      </c>
+      <c r="C69" s="27" t="n"/>
+      <c r="D69" s="27" t="n"/>
+      <c r="E69" s="27" t="n"/>
+      <c r="F69" s="28" t="n"/>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>연간 절감 효과</t>
+        </is>
+      </c>
+      <c r="B70" s="18" t="inlineStr">
+        <is>
+          <t>{{ROI_ANNUAL_SAVE}}</t>
+        </is>
+      </c>
+      <c r="C70" s="27" t="n"/>
+      <c r="D70" s="27" t="n"/>
+      <c r="E70" s="27" t="n"/>
+      <c r="F70" s="28" t="n"/>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>ROI 달성 시점</t>
+        </is>
+      </c>
+      <c r="B71" s="18" t="inlineStr">
+        <is>
+          <t>{{ROI_PAYBACK}}</t>
+        </is>
+      </c>
+      <c r="C71" s="27" t="n"/>
+      <c r="D71" s="27" t="n"/>
+      <c r="E71" s="27" t="n"/>
+      <c r="F71" s="28" t="n"/>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>구축 소요 시간</t>
+        </is>
+      </c>
+      <c r="B72" s="18" t="inlineStr">
+        <is>
+          <t>{{ROI_BUILD_TIME}}</t>
+        </is>
+      </c>
+      <c r="C72" s="27" t="n"/>
+      <c r="D72" s="27" t="n"/>
+      <c r="E72" s="27" t="n"/>
+      <c r="F72" s="28" t="n"/>
+    </row>
+    <row r="74" ht="24" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  부록 A.  재컨설팅 이력</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
         <is>
           <t>Rev</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B75" s="3" t="inlineStr">
         <is>
           <t>타입</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr">
+      <c r="C75" s="3" t="inlineStr">
         <is>
           <t>이전 권고</t>
         </is>
       </c>
-      <c r="D67" s="3" t="inlineStr">
+      <c r="D75" s="3" t="inlineStr">
         <is>
           <t>새 권고</t>
         </is>
       </c>
-      <c r="E67" s="3" t="inlineStr">
+      <c r="E75" s="3" t="inlineStr">
         <is>
           <t>변경 이유</t>
         </is>
       </c>
-      <c r="F67" s="3" t="inlineStr"/>
-    </row>
-    <row r="68" ht="22" customHeight="1">
-      <c r="A68" s="14" t="inlineStr">
+      <c r="F75" s="3" t="inlineStr"/>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="14" t="inlineStr">
         <is>
           <t>{{REV_1_NO}}</t>
         </is>
       </c>
-      <c r="B68" s="14" t="inlineStr">
+      <c r="B76" s="14" t="inlineStr">
         <is>
           <t>{{REV_1_TYPE}}</t>
         </is>
       </c>
-      <c r="C68" s="17" t="inlineStr">
+      <c r="C76" s="19" t="inlineStr">
         <is>
           <t>{{REV_1_PREV}}</t>
         </is>
       </c>
-      <c r="D68" s="17" t="inlineStr">
+      <c r="D76" s="19" t="inlineStr">
         <is>
           <t>{{REV_1_NEW}}</t>
         </is>
       </c>
-      <c r="E68" s="17" t="inlineStr">
+      <c r="E76" s="19" t="inlineStr">
         <is>
           <t>{{REV_1_REASON}}</t>
         </is>
       </c>
-      <c r="F68" s="26" t="n"/>
-    </row>
-    <row r="69" ht="22" customHeight="1">
-      <c r="A69" s="14" t="inlineStr">
+      <c r="F76" s="28" t="n"/>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="14" t="inlineStr">
         <is>
           <t>{{REV_2_NO}}</t>
         </is>
       </c>
-      <c r="B69" s="14" t="inlineStr">
+      <c r="B77" s="14" t="inlineStr">
         <is>
           <t>{{REV_2_TYPE}}</t>
         </is>
       </c>
-      <c r="C69" s="17" t="inlineStr">
+      <c r="C77" s="19" t="inlineStr">
         <is>
           <t>{{REV_2_PREV}}</t>
         </is>
       </c>
-      <c r="D69" s="17" t="inlineStr">
+      <c r="D77" s="19" t="inlineStr">
         <is>
           <t>{{REV_2_NEW}}</t>
         </is>
       </c>
-      <c r="E69" s="17" t="inlineStr">
+      <c r="E77" s="19" t="inlineStr">
         <is>
           <t>{{REV_2_REASON}}</t>
         </is>
       </c>
-      <c r="F69" s="26" t="n"/>
-    </row>
-    <row r="70" ht="22" customHeight="1">
-      <c r="A70" s="14" t="inlineStr">
+      <c r="F77" s="28" t="n"/>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="14" t="inlineStr">
         <is>
           <t>{{REV_3_NO}}</t>
         </is>
       </c>
-      <c r="B70" s="14" t="inlineStr">
+      <c r="B78" s="14" t="inlineStr">
         <is>
           <t>{{REV_3_TYPE}}</t>
         </is>
       </c>
-      <c r="C70" s="17" t="inlineStr">
+      <c r="C78" s="19" t="inlineStr">
         <is>
           <t>{{REV_3_PREV}}</t>
         </is>
       </c>
-      <c r="D70" s="17" t="inlineStr">
+      <c r="D78" s="19" t="inlineStr">
         <is>
           <t>{{REV_3_NEW}}</t>
         </is>
       </c>
-      <c r="E70" s="17" t="inlineStr">
+      <c r="E78" s="19" t="inlineStr">
         <is>
           <t>{{REV_3_REASON}}</t>
         </is>
       </c>
-      <c r="F70" s="26" t="n"/>
-    </row>
-    <row r="71" ht="22" customHeight="1">
-      <c r="A71" s="18" t="inlineStr">
+      <c r="F78" s="28" t="n"/>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="20" t="inlineStr">
         <is>
           <t>총 재컨설팅 횟수: {{REV_TOTAL}}회  (경량: {{REV_LIGHT}}회  |  전체: {{REV_FULL}}회)</t>
         </is>
       </c>
-      <c r="B71" s="25" t="n"/>
-      <c r="C71" s="25" t="n"/>
-      <c r="D71" s="25" t="n"/>
-      <c r="E71" s="25" t="n"/>
-      <c r="F71" s="26" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="19" t="inlineStr">
+      <c r="B79" s="27" t="n"/>
+      <c r="C79" s="27" t="n"/>
+      <c r="D79" s="27" t="n"/>
+      <c r="E79" s="27" t="n"/>
+      <c r="F79" s="28" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="21" t="inlineStr">
         <is>
           <t>※  {{변수명}} 형식의 셀을 실제 데이터로 교체하여 사용합니다.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="53">
+  <mergeCells count="60">
     <mergeCell ref="B62:F62"/>
     <mergeCell ref="A66:F66"/>
-    <mergeCell ref="E68:F68"/>
+    <mergeCell ref="B72:F72"/>
     <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A74:F74"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="B22:F22"/>
     <mergeCell ref="A50:F50"/>
     <mergeCell ref="E48:F48"/>
+    <mergeCell ref="B71:F71"/>
     <mergeCell ref="A55:F55"/>
     <mergeCell ref="B58:F58"/>
     <mergeCell ref="B56:F56"/>
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B52:F52"/>
     <mergeCell ref="B21:F21"/>
-    <mergeCell ref="A71:F71"/>
+    <mergeCell ref="B70:F70"/>
     <mergeCell ref="B43:F43"/>
     <mergeCell ref="B39:F39"/>
     <mergeCell ref="C47:D47"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="B42:F42"/>
     <mergeCell ref="A32:F32"/>
+    <mergeCell ref="B67:F67"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="B23:F23"/>
     <mergeCell ref="B61:F61"/>
-    <mergeCell ref="E69:F69"/>
+    <mergeCell ref="E78:F78"/>
     <mergeCell ref="B57:F57"/>
+    <mergeCell ref="A81:F81"/>
     <mergeCell ref="B53:F53"/>
     <mergeCell ref="B29:F29"/>
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="C46:D46"/>
+    <mergeCell ref="B69:F69"/>
     <mergeCell ref="B38:F38"/>
     <mergeCell ref="E46:F46"/>
     <mergeCell ref="B34:F34"/>
+    <mergeCell ref="E77:F77"/>
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B19:F19"/>
     <mergeCell ref="C48:D48"/>
-    <mergeCell ref="E70:F70"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="B30:F30"/>
-    <mergeCell ref="A73:F73"/>
+    <mergeCell ref="B68:F68"/>
     <mergeCell ref="A2:F3"/>
     <mergeCell ref="A60:F60"/>
     <mergeCell ref="A36:F36"/>
@@ -1839,7 +1961,9 @@
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B33:F33"/>
     <mergeCell ref="B64:F64"/>
+    <mergeCell ref="E76:F76"/>
     <mergeCell ref="B51:F51"/>
+    <mergeCell ref="A79:F79"/>
     <mergeCell ref="B63:F63"/>
     <mergeCell ref="B26:F26"/>
     <mergeCell ref="B41:F41"/>
@@ -1857,7 +1981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:F71"/>
+  <dimension ref="A2:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1870,7 +1994,7 @@
   <sheetData>
     <row r="1" ht="14" customHeight="1"/>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="27" t="inlineStr">
+      <c r="A2" s="29" t="inlineStr">
         <is>
           <t>MS Work Automation  Consulting Report</t>
         </is>
@@ -1879,813 +2003,883 @@
     <row r="3" ht="20" customHeight="1"/>
     <row r="4" ht="6" customHeight="1"/>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  Session Info</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>Session ID</t>
         </is>
       </c>
-      <c r="B6" s="30" t="inlineStr">
+      <c r="B6" s="32" t="inlineStr">
         <is>
           <t>{{SESSION_ID}}</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
+      <c r="C6" s="31" t="inlineStr">
         <is>
           <t>Mode</t>
         </is>
       </c>
-      <c r="D6" s="30" t="inlineStr">
+      <c r="D6" s="32" t="inlineStr">
         <is>
           <t>{{MODE}}</t>
         </is>
       </c>
-      <c r="E6" s="31" t="inlineStr"/>
-      <c r="F6" s="31" t="inlineStr"/>
+      <c r="E6" s="33" t="inlineStr"/>
+      <c r="F6" s="33" t="inlineStr"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="29" t="inlineStr">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t>Created At</t>
         </is>
       </c>
-      <c r="B7" s="30" t="inlineStr">
+      <c r="B7" s="32" t="inlineStr">
         <is>
           <t>{{CREATED_AT}}</t>
         </is>
       </c>
-      <c r="C7" s="29" t="inlineStr">
+      <c r="C7" s="31" t="inlineStr">
         <is>
           <t>Business Domain</t>
         </is>
       </c>
-      <c r="D7" s="30" t="inlineStr">
+      <c r="D7" s="32" t="inlineStr">
         <is>
           <t>{{DOMAIN}}</t>
         </is>
       </c>
-      <c r="E7" s="31" t="inlineStr"/>
-      <c r="F7" s="31" t="inlineStr"/>
+      <c r="E7" s="33" t="inlineStr"/>
+      <c r="F7" s="33" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t>MS Support</t>
         </is>
       </c>
-      <c r="B8" s="30" t="inlineStr">
+      <c r="B8" s="32" t="inlineStr">
         <is>
           <t>{{MS_VERIFY}}</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="31" t="inlineStr">
         <is>
           <t>Parse Confidence</t>
         </is>
       </c>
-      <c r="D8" s="30" t="inlineStr">
+      <c r="D8" s="32" t="inlineStr">
         <is>
           <t>{{PARSE_CONFIDENCE}}%</t>
         </is>
       </c>
-      <c r="E8" s="31" t="inlineStr"/>
-      <c r="F8" s="31" t="inlineStr"/>
+      <c r="E8" s="33" t="inlineStr"/>
+      <c r="F8" s="33" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  1.  Requirements Summary</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Business Domain</t>
         </is>
       </c>
-      <c r="B11" s="30" t="inlineStr">
+      <c r="B11" s="32" t="inlineStr">
         <is>
           <t>{{REQ_DOMAIN}}</t>
         </is>
       </c>
-      <c r="C11" s="29" t="inlineStr">
+      <c r="C11" s="31" t="inlineStr">
         <is>
           <t>Process Type</t>
         </is>
       </c>
-      <c r="D11" s="30" t="inlineStr">
+      <c r="D11" s="32" t="inlineStr">
         <is>
           <t>{{REQ_PROCESS_TYPE}}</t>
         </is>
       </c>
-      <c r="E11" s="31" t="inlineStr"/>
-      <c r="F11" s="31" t="inlineStr"/>
+      <c r="E11" s="33" t="inlineStr"/>
+      <c r="F11" s="33" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>Automation Target</t>
         </is>
       </c>
-      <c r="B12" s="30" t="inlineStr">
+      <c r="B12" s="32" t="inlineStr">
         <is>
           <t>{{REQ_TARGET}}</t>
         </is>
       </c>
-      <c r="C12" s="29" t="inlineStr">
+      <c r="C12" s="31" t="inlineStr">
         <is>
           <t>Send Volume</t>
         </is>
       </c>
-      <c r="D12" s="30" t="inlineStr">
+      <c r="D12" s="32" t="inlineStr">
         <is>
           <t>{{REQ_SCALE}}</t>
         </is>
       </c>
-      <c r="E12" s="31" t="inlineStr"/>
-      <c r="F12" s="31" t="inlineStr"/>
+      <c r="E12" s="33" t="inlineStr"/>
+      <c r="F12" s="33" t="inlineStr"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>Current Tools</t>
         </is>
       </c>
-      <c r="B13" s="30" t="inlineStr">
+      <c r="B13" s="32" t="inlineStr">
         <is>
           <t>{{REQ_CURRENT_TOOL}}</t>
         </is>
       </c>
-      <c r="C13" s="29" t="inlineStr">
+      <c r="C13" s="31" t="inlineStr">
         <is>
           <t>Attachments</t>
         </is>
       </c>
-      <c r="D13" s="30" t="inlineStr">
+      <c r="D13" s="32" t="inlineStr">
         <is>
           <t>{{REQ_ATTACHMENT}}</t>
         </is>
       </c>
-      <c r="E13" s="31" t="inlineStr"/>
-      <c r="F13" s="31" t="inlineStr"/>
+      <c r="E13" s="33" t="inlineStr"/>
+      <c r="F13" s="33" t="inlineStr"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="29" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>External Systems</t>
         </is>
       </c>
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B14" s="32" t="inlineStr">
         <is>
           <t>{{REQ_EXT_SYSTEM}}</t>
         </is>
       </c>
-      <c r="C14" s="29" t="inlineStr">
+      <c r="C14" s="31" t="inlineStr">
         <is>
           <t>History Logging</t>
         </is>
       </c>
-      <c r="D14" s="30" t="inlineStr">
+      <c r="D14" s="32" t="inlineStr">
         <is>
           <t>{{REQ_HISTORY_SAVE}}</t>
         </is>
       </c>
-      <c r="E14" s="31" t="inlineStr"/>
-      <c r="F14" s="31" t="inlineStr"/>
+      <c r="E14" s="33" t="inlineStr"/>
+      <c r="F14" s="33" t="inlineStr"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>Constraints</t>
         </is>
       </c>
-      <c r="B15" s="30" t="inlineStr">
+      <c r="B15" s="32" t="inlineStr">
         <is>
           <t>{{REQ_CONSTRAINTS}}</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="32" t="inlineStr">
+      <c r="A17" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  2.  User-Facing Solution Guide</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="33" t="inlineStr">
+      <c r="A18" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">  [ Recommended ]   {{SOL_REC_NAME}}</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="29" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>Solution Name</t>
         </is>
       </c>
-      <c r="B19" s="34" t="inlineStr">
+      <c r="B19" s="36" t="inlineStr">
         <is>
           <t>{{SOL_REC_NAME}}</t>
         </is>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>Recommendation Reason</t>
         </is>
       </c>
-      <c r="B20" s="34" t="inlineStr">
+      <c r="B20" s="36" t="inlineStr">
         <is>
           <t>{{SOL_REC_REASON}}</t>
         </is>
       </c>
     </row>
     <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="29" t="inlineStr">
+      <c r="A21" s="31" t="inlineStr">
         <is>
           <t>Implementation Flow</t>
         </is>
       </c>
-      <c r="B21" s="34" t="inlineStr">
+      <c r="B21" s="36" t="inlineStr">
         <is>
           <t>{{SOL_REC_FLOW}}</t>
         </is>
       </c>
     </row>
     <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="29" t="inlineStr">
+      <c r="A22" s="31" t="inlineStr">
         <is>
           <t>Prerequisites</t>
         </is>
       </c>
-      <c r="B22" s="34" t="inlineStr">
+      <c r="B22" s="36" t="inlineStr">
         <is>
           <t>{{SOL_REC_PREREQ}}</t>
         </is>
       </c>
     </row>
     <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="29" t="inlineStr">
+      <c r="A23" s="31" t="inlineStr">
         <is>
           <t>Cautions</t>
         </is>
       </c>
-      <c r="B23" s="34" t="inlineStr">
+      <c r="B23" s="36" t="inlineStr">
         <is>
           <t>{{SOL_REC_CAUTION}}</t>
         </is>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="35" t="inlineStr">
+      <c r="A25" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">  [ Needs Review ]   {{SOL_REV_NAME}}</t>
         </is>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="29" t="inlineStr">
+      <c r="A26" s="31" t="inlineStr">
         <is>
           <t>Solution Name</t>
         </is>
       </c>
-      <c r="B26" s="36" t="inlineStr">
+      <c r="B26" s="38" t="inlineStr">
         <is>
           <t>{{SOL_REV_NAME}}</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="29" t="inlineStr">
+      <c r="A27" s="31" t="inlineStr">
         <is>
           <t>Reason / Limitation</t>
         </is>
       </c>
-      <c r="B27" s="36" t="inlineStr">
+      <c r="B27" s="38" t="inlineStr">
         <is>
           <t>{{SOL_REV_REASON}}</t>
         </is>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="29" t="inlineStr">
+      <c r="A28" s="31" t="inlineStr">
         <is>
           <t>Judgment Basis</t>
         </is>
       </c>
-      <c r="B28" s="36" t="inlineStr">
+      <c r="B28" s="38" t="inlineStr">
         <is>
           <t>{{SOL_REV_JUDGMENT}}</t>
         </is>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="37" t="inlineStr">
+      <c r="A30" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">  [ Not Recommended ]   {{SOL_NOT_NAME}}</t>
         </is>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="29" t="inlineStr">
+      <c r="A31" s="31" t="inlineStr">
         <is>
           <t>Solution Name</t>
         </is>
       </c>
-      <c r="B31" s="38" t="inlineStr">
+      <c r="B31" s="40" t="inlineStr">
         <is>
           <t>{{SOL_NOT_NAME}}</t>
         </is>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="29" t="inlineStr">
+      <c r="A32" s="31" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="B32" s="38" t="inlineStr">
+      <c r="B32" s="40" t="inlineStr">
         <is>
           <t>{{SOL_NOT_REASON}}</t>
         </is>
       </c>
     </row>
     <row r="34" ht="24" customHeight="1">
-      <c r="A34" s="32" t="inlineStr">
+      <c r="A34" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  3.  Developer Technical Specification</t>
         </is>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="33" t="inlineStr">
+      <c r="A35" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">  [ Recommended ]   {{SOL_REC_NAME}}</t>
         </is>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="29" t="inlineStr">
+      <c r="A36" s="31" t="inlineStr">
         <is>
           <t>Solution Name / ID</t>
         </is>
       </c>
-      <c r="B36" s="34" t="inlineStr">
+      <c r="B36" s="36" t="inlineStr">
         <is>
           <t>{{SOL_REC_NAME}}  |  ID: {{SOL_REC_ID}}</t>
         </is>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="29" t="inlineStr">
+      <c r="A37" s="31" t="inlineStr">
         <is>
           <t>Rationale</t>
         </is>
       </c>
-      <c r="B37" s="34" t="inlineStr">
+      <c r="B37" s="36" t="inlineStr">
         <is>
           <t>{{SOL_REC_TECH_REASON}}</t>
         </is>
       </c>
     </row>
     <row r="38" ht="50" customHeight="1">
-      <c r="A38" s="29" t="inlineStr">
+      <c r="A38" s="31" t="inlineStr">
         <is>
           <t>Implementation Overview</t>
         </is>
       </c>
-      <c r="B38" s="34" t="inlineStr">
+      <c r="B38" s="36" t="inlineStr">
         <is>
           <t>{{SOL_REC_IMPL_OVERVIEW}}</t>
         </is>
       </c>
     </row>
     <row r="39" ht="50" customHeight="1">
-      <c r="A39" s="29" t="inlineStr">
+      <c r="A39" s="31" t="inlineStr">
         <is>
           <t>Prerequisites</t>
         </is>
       </c>
-      <c r="B39" s="34" t="inlineStr">
+      <c r="B39" s="36" t="inlineStr">
         <is>
           <t>{{SOL_REC_PREREQ_TECH}}</t>
         </is>
       </c>
     </row>
     <row r="40" ht="50" customHeight="1">
-      <c r="A40" s="29" t="inlineStr">
+      <c r="A40" s="31" t="inlineStr">
         <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="B40" s="34" t="inlineStr">
+      <c r="B40" s="36" t="inlineStr">
         <is>
           <t>{{SOL_REC_LIMITS}}</t>
         </is>
       </c>
     </row>
     <row r="41" ht="50" customHeight="1">
-      <c r="A41" s="29" t="inlineStr">
+      <c r="A41" s="31" t="inlineStr">
         <is>
           <t>Considerations</t>
         </is>
       </c>
-      <c r="B41" s="34" t="inlineStr">
+      <c r="B41" s="36" t="inlineStr">
         <is>
           <t>{{SOL_REC_CONSIDERATIONS}}</t>
         </is>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="29" t="inlineStr">
+      <c r="A42" s="31" t="inlineStr">
         <is>
           <t>Risk Details</t>
         </is>
       </c>
-      <c r="B42" s="31" t="inlineStr"/>
-      <c r="C42" s="31" t="inlineStr"/>
-      <c r="D42" s="31" t="inlineStr"/>
-      <c r="E42" s="31" t="inlineStr"/>
-      <c r="F42" s="31" t="inlineStr"/>
+      <c r="B42" s="33" t="inlineStr"/>
+      <c r="C42" s="33" t="inlineStr"/>
+      <c r="D42" s="33" t="inlineStr"/>
+      <c r="E42" s="33" t="inlineStr"/>
+      <c r="F42" s="33" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="29" t="inlineStr">
+      <c r="A43" s="31" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B43" s="29" t="inlineStr">
+      <c r="B43" s="31" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="C43" s="29" t="inlineStr">
-        <is>
-          <t>Trigger Condition</t>
-        </is>
-      </c>
-      <c r="D43" s="29" t="inlineStr">
-        <is>
-          <t>Mitigation</t>
-        </is>
-      </c>
-      <c r="E43" s="31" t="inlineStr"/>
-      <c r="F43" s="31" t="inlineStr"/>
+      <c r="C43" s="33" t="inlineStr"/>
+      <c r="D43" s="33" t="inlineStr"/>
+      <c r="E43" s="33" t="inlineStr"/>
+      <c r="F43" s="33" t="inlineStr"/>
     </row>
     <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="39" t="inlineStr">
+      <c r="A44" s="41" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="B44" s="40" t="inlineStr">
+      <c r="B44" s="42" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="C44" s="30" t="inlineStr">
+      <c r="C44" s="32" t="inlineStr">
         <is>
           <t>{{RISK_SEC_CONDITION}}</t>
         </is>
       </c>
-      <c r="E44" s="30" t="inlineStr">
+      <c r="E44" s="32" t="inlineStr">
         <is>
           <t>{{RISK_SEC_ACTION}}</t>
         </is>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="39" t="inlineStr">
+      <c r="A45" s="41" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="B45" s="40" t="inlineStr">
+      <c r="B45" s="42" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="C45" s="30" t="inlineStr">
+      <c r="C45" s="32" t="inlineStr">
         <is>
           <t>{{RISK_LIC_CONDITION}}</t>
         </is>
       </c>
-      <c r="E45" s="30" t="inlineStr">
+      <c r="E45" s="32" t="inlineStr">
         <is>
           <t>{{RISK_LIC_ACTION}}</t>
         </is>
       </c>
     </row>
     <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="39" t="inlineStr">
+      <c r="A46" s="41" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="B46" s="40" t="inlineStr">
+      <c r="B46" s="42" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="C46" s="30" t="inlineStr">
+      <c r="C46" s="32" t="inlineStr">
         <is>
           <t>{{RISK_OPS_CONDITION}}</t>
         </is>
       </c>
-      <c r="E46" s="30" t="inlineStr">
+      <c r="E46" s="32" t="inlineStr">
         <is>
           <t>{{RISK_OPS_ACTION}}</t>
         </is>
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="35" t="inlineStr">
+      <c r="A48" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">  [ Needs Review ]   {{SOL_REV_NAME}}</t>
         </is>
       </c>
     </row>
     <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="29" t="inlineStr">
+      <c r="A49" s="31" t="inlineStr">
         <is>
           <t>Solution Name / ID</t>
         </is>
       </c>
-      <c r="B49" s="36" t="inlineStr">
+      <c r="B49" s="38" t="inlineStr">
         <is>
           <t>{{SOL_REV_NAME}}  |  ID: {{SOL_REV_ID}}</t>
         </is>
       </c>
     </row>
     <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="29" t="inlineStr">
+      <c r="A50" s="31" t="inlineStr">
         <is>
           <t>Rationale</t>
         </is>
       </c>
-      <c r="B50" s="36" t="inlineStr">
+      <c r="B50" s="38" t="inlineStr">
         <is>
           <t>{{SOL_REV_TECH_REASON}}</t>
         </is>
       </c>
     </row>
     <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="29" t="inlineStr">
+      <c r="A51" s="31" t="inlineStr">
         <is>
           <t>Judgment Basis</t>
         </is>
       </c>
-      <c r="B51" s="36" t="inlineStr">
+      <c r="B51" s="38" t="inlineStr">
         <is>
           <t>{{SOL_REV_JUDGMENT}}</t>
         </is>
       </c>
     </row>
     <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="37" t="inlineStr">
+      <c r="A53" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">  [ Not Recommended ]   {{SOL_NOT_NAME}}</t>
         </is>
       </c>
     </row>
     <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="29" t="inlineStr">
+      <c r="A54" s="31" t="inlineStr">
         <is>
           <t>Solution Name / ID</t>
         </is>
       </c>
-      <c r="B54" s="38" t="inlineStr">
+      <c r="B54" s="40" t="inlineStr">
         <is>
           <t>{{SOL_NOT_NAME}}  |  ID: {{SOL_NOT_ID}}</t>
         </is>
       </c>
     </row>
     <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="29" t="inlineStr">
+      <c r="A55" s="31" t="inlineStr">
         <is>
           <t>Rationale</t>
         </is>
       </c>
-      <c r="B55" s="38" t="inlineStr">
+      <c r="B55" s="40" t="inlineStr">
         <is>
           <t>{{SOL_NOT_TECH_REASON}}</t>
         </is>
       </c>
     </row>
     <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="29" t="inlineStr">
+      <c r="A56" s="31" t="inlineStr">
         <is>
           <t>Judgment Basis</t>
         </is>
       </c>
-      <c r="B56" s="38" t="inlineStr">
+      <c r="B56" s="40" t="inlineStr">
         <is>
           <t>{{SOL_NOT_JUDGMENT}}</t>
         </is>
       </c>
     </row>
     <row r="58" ht="24" customHeight="1">
-      <c r="A58" s="41" t="inlineStr">
+      <c r="A58" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">  4.  AI Deep Analysis</t>
         </is>
       </c>
     </row>
     <row r="59" ht="50" customHeight="1">
-      <c r="A59" s="29" t="inlineStr">
+      <c r="A59" s="31" t="inlineStr">
         <is>
           <t>Analysis Overview</t>
         </is>
       </c>
-      <c r="B59" s="42" t="inlineStr">
+      <c r="B59" s="44" t="inlineStr">
         <is>
           <t>{{AI_OVERVIEW}}</t>
         </is>
       </c>
     </row>
     <row r="60" ht="50" customHeight="1">
-      <c r="A60" s="29" t="inlineStr">
+      <c r="A60" s="31" t="inlineStr">
         <is>
           <t>Key Findings</t>
         </is>
       </c>
-      <c r="B60" s="42" t="inlineStr">
+      <c r="B60" s="44" t="inlineStr">
         <is>
           <t>{{AI_FINDINGS}}</t>
         </is>
       </c>
     </row>
     <row r="61" ht="50" customHeight="1">
-      <c r="A61" s="29" t="inlineStr">
+      <c r="A61" s="31" t="inlineStr">
         <is>
           <t>Optimization Recommendations</t>
         </is>
       </c>
-      <c r="B61" s="42" t="inlineStr">
+      <c r="B61" s="44" t="inlineStr">
         <is>
           <t>{{AI_RECOMMENDATIONS}}</t>
         </is>
       </c>
     </row>
     <row r="62" ht="50" customHeight="1">
-      <c r="A62" s="29" t="inlineStr">
+      <c r="A62" s="31" t="inlineStr">
         <is>
           <t>Additional Risks / Opportunities</t>
         </is>
       </c>
-      <c r="B62" s="42" t="inlineStr">
+      <c r="B62" s="44" t="inlineStr">
         <is>
           <t>{{AI_EXTRA_RISK_OPP}}</t>
         </is>
       </c>
     </row>
     <row r="64" ht="24" customHeight="1">
-      <c r="A64" s="28" t="inlineStr">
+      <c r="A64" s="45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5.  ROI Estimation</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="31" t="inlineStr">
+        <is>
+          <t>Current Work Time</t>
+        </is>
+      </c>
+      <c r="B65" s="46" t="inlineStr">
+        <is>
+          <t>{{ROI_CURRENT_TIME}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="31" t="inlineStr">
+        <is>
+          <t>Improved Work Time</t>
+        </is>
+      </c>
+      <c r="B66" s="46" t="inlineStr">
+        <is>
+          <t>{{ROI_IMPROVED_TIME}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="31" t="inlineStr">
+        <is>
+          <t>Time Saved (per unit)</t>
+        </is>
+      </c>
+      <c r="B67" s="46" t="inlineStr">
+        <is>
+          <t>{{ROI_SAVE_PERIOD}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="31" t="inlineStr">
+        <is>
+          <t>Annual Time Saved</t>
+        </is>
+      </c>
+      <c r="B68" s="46" t="inlineStr">
+        <is>
+          <t>{{ROI_ANNUAL_SAVE}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="31" t="inlineStr">
+        <is>
+          <t>ROI Payback Period</t>
+        </is>
+      </c>
+      <c r="B69" s="46" t="inlineStr">
+        <is>
+          <t>{{ROI_PAYBACK}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="31" t="inlineStr">
+        <is>
+          <t>Build Time Required</t>
+        </is>
+      </c>
+      <c r="B70" s="46" t="inlineStr">
+        <is>
+          <t>{{ROI_BUILD_TIME}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="24" customHeight="1">
+      <c r="A72" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  Appendix A.  Revision History</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="29" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="31" t="inlineStr">
         <is>
           <t>Rev</t>
         </is>
       </c>
-      <c r="B65" s="29" t="inlineStr">
+      <c r="B73" s="31" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C65" s="29" t="inlineStr">
+      <c r="C73" s="31" t="inlineStr">
         <is>
           <t>Previous Recommendation</t>
         </is>
       </c>
-      <c r="D65" s="29" t="inlineStr">
+      <c r="D73" s="31" t="inlineStr">
         <is>
           <t>New Recommendation</t>
         </is>
       </c>
-      <c r="E65" s="29" t="inlineStr">
+      <c r="E73" s="31" t="inlineStr">
         <is>
           <t>Reason for Change</t>
         </is>
       </c>
-      <c r="F65" s="29" t="inlineStr"/>
-    </row>
-    <row r="66" ht="22" customHeight="1">
-      <c r="A66" s="40" t="inlineStr">
+      <c r="F73" s="31" t="inlineStr"/>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="42" t="inlineStr">
         <is>
           <t>{{REV_1_NO}}</t>
         </is>
       </c>
-      <c r="B66" s="40" t="inlineStr">
+      <c r="B74" s="42" t="inlineStr">
         <is>
           <t>{{REV_1_TYPE}}</t>
         </is>
       </c>
-      <c r="C66" s="43" t="inlineStr">
+      <c r="C74" s="47" t="inlineStr">
         <is>
           <t>{{REV_1_PREV}}</t>
         </is>
       </c>
-      <c r="D66" s="43" t="inlineStr">
+      <c r="D74" s="47" t="inlineStr">
         <is>
           <t>{{REV_1_NEW}}</t>
         </is>
       </c>
-      <c r="E66" s="43" t="inlineStr">
+      <c r="E74" s="47" t="inlineStr">
         <is>
           <t>{{REV_1_REASON}}</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="22" customHeight="1">
-      <c r="A67" s="40" t="inlineStr">
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="42" t="inlineStr">
         <is>
           <t>{{REV_2_NO}}</t>
         </is>
       </c>
-      <c r="B67" s="40" t="inlineStr">
+      <c r="B75" s="42" t="inlineStr">
         <is>
           <t>{{REV_2_TYPE}}</t>
         </is>
       </c>
-      <c r="C67" s="43" t="inlineStr">
+      <c r="C75" s="47" t="inlineStr">
         <is>
           <t>{{REV_2_PREV}}</t>
         </is>
       </c>
-      <c r="D67" s="43" t="inlineStr">
+      <c r="D75" s="47" t="inlineStr">
         <is>
           <t>{{REV_2_NEW}}</t>
         </is>
       </c>
-      <c r="E67" s="43" t="inlineStr">
+      <c r="E75" s="47" t="inlineStr">
         <is>
           <t>{{REV_2_REASON}}</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="22" customHeight="1">
-      <c r="A68" s="40" t="inlineStr">
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="42" t="inlineStr">
         <is>
           <t>{{REV_3_NO}}</t>
         </is>
       </c>
-      <c r="B68" s="40" t="inlineStr">
+      <c r="B76" s="42" t="inlineStr">
         <is>
           <t>{{REV_3_TYPE}}</t>
         </is>
       </c>
-      <c r="C68" s="43" t="inlineStr">
+      <c r="C76" s="47" t="inlineStr">
         <is>
           <t>{{REV_3_PREV}}</t>
         </is>
       </c>
-      <c r="D68" s="43" t="inlineStr">
+      <c r="D76" s="47" t="inlineStr">
         <is>
           <t>{{REV_3_NEW}}</t>
         </is>
       </c>
-      <c r="E68" s="43" t="inlineStr">
+      <c r="E76" s="47" t="inlineStr">
         <is>
           <t>{{REV_3_REASON}}</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="22" customHeight="1">
-      <c r="A69" s="44" t="inlineStr">
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="48" t="inlineStr">
         <is>
           <t>Total Revisions: {{REV_TOTAL}}  (Light: {{REV_LIGHT}}  |  Full: {{REV_FULL}})</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="45" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="49" t="inlineStr">
         <is>
           <t>Note: Replace all {{VARIABLE_NAME}} cells with actual data before use.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="51">
+  <mergeCells count="58">
     <mergeCell ref="B54:F54"/>
     <mergeCell ref="B62:F62"/>
-    <mergeCell ref="E68:F68"/>
     <mergeCell ref="B59:F59"/>
-    <mergeCell ref="E67:F67"/>
+    <mergeCell ref="B66:F66"/>
     <mergeCell ref="C45:D45"/>
     <mergeCell ref="B31:F31"/>
     <mergeCell ref="A18:F18"/>
@@ -2693,20 +2887,23 @@
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B56:F56"/>
     <mergeCell ref="E44:F44"/>
+    <mergeCell ref="B70:F70"/>
     <mergeCell ref="B21:F21"/>
-    <mergeCell ref="A71:F71"/>
     <mergeCell ref="B39:F39"/>
-    <mergeCell ref="A69:F69"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="B60:F60"/>
+    <mergeCell ref="B67:F67"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="B23:F23"/>
     <mergeCell ref="A35:F35"/>
     <mergeCell ref="B61:F61"/>
     <mergeCell ref="A53:F53"/>
+    <mergeCell ref="A72:F72"/>
+    <mergeCell ref="E74:F74"/>
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="C46:D46"/>
+    <mergeCell ref="B69:F69"/>
     <mergeCell ref="B38:F38"/>
     <mergeCell ref="E46:F46"/>
     <mergeCell ref="B28:F28"/>
@@ -2717,15 +2914,20 @@
     <mergeCell ref="A34:F34"/>
     <mergeCell ref="A48:F48"/>
     <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A77:F77"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="A64:F64"/>
     <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B65:F65"/>
+    <mergeCell ref="B68:F68"/>
     <mergeCell ref="A2:F3"/>
     <mergeCell ref="B55:F55"/>
+    <mergeCell ref="E76:F76"/>
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B51:F51"/>
-    <mergeCell ref="E66:F66"/>
+    <mergeCell ref="A79:F79"/>
+    <mergeCell ref="E75:F75"/>
     <mergeCell ref="B36:F36"/>
     <mergeCell ref="B32:F32"/>
     <mergeCell ref="B50:F50"/>

</xml_diff>